<commit_message>
Regenerar pricing y dashboard tras cancelación Derek Stray
Huecos jun 16-19 y jun 22-24 ahora visibles en Revenue Cockpit.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -51,12 +51,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8DAEF"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E8DAEF"/>
       </patternFill>
     </fill>
   </fills>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="51" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>86.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>56.48</v>
@@ -648,31 +648,27 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>56.94</v>
+        <v>56.82</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>51.25</v>
+        <v>51.14</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
+      <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-05-23; sin vender → precio Ocupación</t>
+          <t>Hueco próximo — revisar diariamente</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -683,110 +679,106 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>88.90000000000001</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>75.11</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>78.67</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>82.33</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (81€–82€)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>81.81</v>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>81.95999999999999</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>73.76000000000001</v>
-      </c>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-05-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>75.11</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>93.03</v>
+      <c r="F3" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>78.38</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>82.12</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (74€–77€)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>baja antelación (↓10%) + hueco corto (↓5%) + ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>67.87</v>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco corto (↓5%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-01; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>92.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -794,7 +786,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -803,278 +795,274 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>88.90000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>92.25</v>
+        <v>74.25</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>100.41</v>
+        <v>78.38</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>105.03</v>
+        <v>82.12</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad</t>
+          <t>Equilibrio</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P65–P75  (104€–105€)</t>
+          <t>P45–P60  (78€–79€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>104.64</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>104.9</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>94.41</v>
+        <v>70.84</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
+          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-07; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>78.38</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>82.12</v>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>P65–P75  (81€–82€)</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>81.56</v>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>81.56</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-05-29; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>100.41</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>105.03</v>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>P65–P75  (104€–105€)</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>104.64</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>94.31999999999999</v>
+      </c>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>Revisar 2026-06-10; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="W6" s="4" t="n">
         <v>92.25</v>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="X6" s="4" t="n">
         <v>118.68</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>92.25</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>100.41</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>105.03</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (104€–105€)</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>104.64</v>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>105</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="U5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="V5" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W5" s="3" t="n">
-        <v>92.25</v>
-      </c>
-      <c r="X5" s="3" t="n">
-        <v>118.68</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>84</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>99</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>105</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–105€)</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>103.5</v>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>104.25</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>93.83</v>
-      </c>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="X6" s="3" t="n">
-        <v>118.65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1082,7 +1070,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1091,366 +1079,558 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>52.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>93.75</v>
+        <v>92.25</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>99</v>
+        <v>100.41</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>105</v>
+        <v>105.03</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Equilibrio</t>
+          <t>Rentabilidad</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>P45–P60  (97€–100€)</t>
+          <t>P65–P75  (104€–105€)</t>
         </is>
       </c>
       <c r="M7" s="4" t="n">
-        <v>98.86</v>
+        <v>104.64</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O7" s="4" t="n">
-        <v>99.31999999999999</v>
+        <v>104.8</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>89.39</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>118.68</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>105.81</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–106€)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%)</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>104.47</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>94.02</v>
+      </c>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%).</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>119.57</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>105.81</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (97€–100€)</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>98.86</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>89.11</v>
+      </c>
+      <c r="Q9" s="3" t="n"/>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="U9" s="3" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
+      <c r="V9" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W7" s="4" t="n">
+      <c r="W9" s="3" t="n">
         <v>93.75</v>
       </c>
-      <c r="X7" s="4" t="n">
-        <v>118.65</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="X9" s="3" t="n">
+        <v>119.57</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>133</v>
-      </c>
-      <c r="G8" s="2" t="n">
+      <c r="F10" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>26.7</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I10" s="2" t="n">
         <v>60.1</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J10" s="2" t="n">
         <v>66.44</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M10" s="2" t="n">
         <v>53.92</v>
       </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>48.69</v>
-      </c>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>48.36</v>
+      </c>
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W8" s="2" t="n">
+      <c r="W10" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="X8" s="2" t="n">
+      <c r="X10" s="2" t="n">
         <v>75.08</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C11" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>143</v>
-      </c>
-      <c r="G9" s="4" t="n">
+      <c r="F11" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>17.8</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H11" s="3" t="n">
         <v>52.08</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I11" s="3" t="n">
         <v>60.1</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J11" s="3" t="n">
         <v>66.44</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (57€–61€)</t>
         </is>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="M11" s="3" t="n">
         <v>59.16</v>
       </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q9" s="4" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>59.37</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>53.43</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>394.81</v>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr">
+      <c r="U11" s="3" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
+      <c r="V11" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W9" s="4" t="n">
+      <c r="W11" s="3" t="n">
         <v>52.08</v>
       </c>
-      <c r="X9" s="4" t="n">
+      <c r="X11" s="3" t="n">
         <v>75.08</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C12" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>163</v>
-      </c>
-      <c r="G10" s="4" t="n">
+      <c r="F12" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="G12" s="3" t="n">
         <v>11.1</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H12" s="3" t="n">
         <v>43.9</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I12" s="3" t="n">
         <v>47.75</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J12" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
-      <c r="M10" s="4" t="n">
+      <c r="M12" s="3" t="n">
         <v>48.17</v>
       </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>43.56</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>321.86</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S10" s="4" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>321.19</v>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="U10" s="4" t="inlineStr">
+      <c r="U12" s="3" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
+      <c r="V12" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W10" s="4" t="n">
+      <c r="W12" s="3" t="n">
         <v>43.9</v>
       </c>
-      <c r="X10" s="4" t="n">
+      <c r="X12" s="3" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1582,25 +1762,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38.08</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>39.88</v>
+        <v>40.67</v>
       </c>
       <c r="D3" t="n">
-        <v>40.82</v>
+        <v>41</v>
       </c>
       <c r="E3" t="n">
         <v>41</v>
       </c>
       <c r="F3" t="n">
-        <v>41.77</v>
+        <v>42.14</v>
       </c>
       <c r="G3" t="n">
-        <v>42.78</v>
+        <v>43.12</v>
       </c>
       <c r="H3" t="n">
-        <v>45.6</v>
+        <v>45.88</v>
       </c>
       <c r="I3" t="n">
         <v>35.5</v>
@@ -1609,7 +1789,7 @@
         <v>50.67</v>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -1619,25 +1799,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>43.39</v>
+        <v>44.56</v>
       </c>
       <c r="C4" t="n">
-        <v>46.5</v>
+        <v>47.25</v>
       </c>
       <c r="D4" t="n">
-        <v>47.81</v>
+        <v>47.95</v>
       </c>
       <c r="E4" t="n">
-        <v>48.1</v>
+        <v>48.2</v>
       </c>
       <c r="F4" t="n">
-        <v>49.33</v>
+        <v>49.4</v>
       </c>
       <c r="G4" t="n">
-        <v>49.66</v>
+        <v>49.87</v>
       </c>
       <c r="H4" t="n">
-        <v>50.88</v>
+        <v>51</v>
       </c>
       <c r="I4" t="n">
         <v>36</v>
@@ -1646,7 +1826,7 @@
         <v>60.33</v>
       </c>
       <c r="K4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -1730,34 +1910,34 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>75.11</v>
+        <v>74.25</v>
       </c>
       <c r="C7" t="n">
-        <v>78.06999999999999</v>
+        <v>76.83</v>
       </c>
       <c r="D7" t="n">
+        <v>78.02</v>
+      </c>
+      <c r="E7" t="n">
         <v>78.38</v>
       </c>
-      <c r="E7" t="n">
-        <v>78.67</v>
-      </c>
       <c r="F7" t="n">
-        <v>79.48</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>81.28</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>82.33</v>
+        <v>82.12</v>
       </c>
       <c r="I7" t="n">
-        <v>70.5</v>
+        <v>35.43</v>
       </c>
       <c r="J7" t="n">
         <v>105.07</v>
       </c>
       <c r="K7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -1822,7 +2002,7 @@
         <v>102</v>
       </c>
       <c r="H9" t="n">
-        <v>105</v>
+        <v>105.81</v>
       </c>
       <c r="I9" t="n">
         <v>73</v>
@@ -2057,7 +2237,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2273,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.045 (auto — vs 1.045 auto)</t>
+          <t>1.015 (auto — vs 1.015 auto)</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2285,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.045</t>
+          <t>1.015</t>
         </is>
       </c>
     </row>
@@ -2322,12 +2502,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 10:53:13</t>
+          <t>2026-05-29 10:11:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2342,17 +2522,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.045</t>
+          <t>1.015</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.045</t>
+          <t>1.015</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Dos reservas nuevas jun 2026 (Vicent + Janine NRF) + Janine rate_type corregida
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -622,7 +622,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>81.09999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>56.48</v>
@@ -648,19 +648,19 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>56.82</v>
+        <v>56.94</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>51.14</v>
+        <v>51.25</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -681,7 +681,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -703,19 +703,19 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>84.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>78.38</v>
+        <v>78.67</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>82.12</v>
+        <v>82.42</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -724,50 +724,50 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>P25–P40  (74€–77€)</t>
+          <t>P25–P40  (75€–78€)</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>75.54000000000001</v>
+        <v>76.53</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + hueco corto (↓5%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>75.41</v>
+        <v>76.53</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>67.87</v>
+        <v>68.88</v>
       </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco corto (↓5%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-01; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-06-03; sin vender → bajar 5–10%</t>
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>74.25</v>
+        <v>67.55</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>92.8</v>
+        <v>93.13</v>
       </c>
     </row>
     <row r="4">
@@ -801,13 +801,13 @@
         <v>86.7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>78.38</v>
+        <v>78.67</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>82.12</v>
+        <v>82.42</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -816,27 +816,27 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (78€–79€)</t>
+          <t>P45–P60  (78€–81€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>78.70999999999999</v>
+        <v>79.81</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>78.70999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>70.84</v>
+        <v>72.09</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S4" s="3" t="n"/>
@@ -856,10 +856,10 @@
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>92.8</v>
+        <v>93.13</v>
       </c>
     </row>
     <row r="5">
@@ -893,13 +893,13 @@
         <v>88.90000000000001</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>78.38</v>
+        <v>78.67</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>82.12</v>
+        <v>82.42</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -912,23 +912,23 @@
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>81.56</v>
+        <v>81.94</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
-        <v>81.56</v>
+        <v>82.05</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>73.40000000000001</v>
+        <v>73.84</v>
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
@@ -952,10 +952,10 @@
         </is>
       </c>
       <c r="W5" s="4" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="X5" s="4" t="n">
-        <v>92.8</v>
+        <v>93.13</v>
       </c>
     </row>
     <row r="6">
@@ -1012,19 +1012,19 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>104.8</v>
+        <v>104.9</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>94.31999999999999</v>
+        <v>94.41</v>
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O7" s="4" t="n">
-        <v>104.8</v>
+        <v>104.9</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>94.31999999999999</v>
+        <v>94.41</v>
       </c>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
@@ -1204,19 +1204,19 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
         </is>
       </c>
       <c r="O8" s="4" t="n">
-        <v>104.47</v>
+        <v>104.85</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>94.02</v>
+        <v>94.36</v>
       </c>
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
@@ -1300,19 +1300,19 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O9" s="3" t="n">
-        <v>99.01000000000001</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>89.11</v>
+        <v>89.39</v>
       </c>
       <c r="Q9" s="3" t="n"/>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
@@ -1396,19 +1396,19 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>53.73</v>
+        <v>54.1</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>48.36</v>
+        <v>48.69</v>
       </c>
       <c r="Q10" s="2" t="n"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1492,21 +1492,21 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O11" s="3" t="n">
-        <v>59.37</v>
+        <v>59.8</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>53.43</v>
+        <v>53.82</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>394.81</v>
+        <v>397.67</v>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr">
@@ -1590,21 +1590,21 @@
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O12" s="3" t="n">
-        <v>48.3</v>
+        <v>48.4</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>43.47</v>
+        <v>43.56</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>321.19</v>
+        <v>321.86</v>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr">
@@ -1910,25 +1910,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>74.25</v>
+        <v>75.06</v>
       </c>
       <c r="C7" t="n">
-        <v>76.83</v>
+        <v>78</v>
       </c>
       <c r="D7" t="n">
-        <v>78.02</v>
+        <v>78.38</v>
       </c>
       <c r="E7" t="n">
-        <v>78.38</v>
+        <v>78.67</v>
       </c>
       <c r="F7" t="n">
-        <v>79.40000000000001</v>
+        <v>81.25</v>
       </c>
       <c r="G7" t="n">
-        <v>80.98999999999999</v>
+        <v>81.45</v>
       </c>
       <c r="H7" t="n">
-        <v>82.12</v>
+        <v>82.42</v>
       </c>
       <c r="I7" t="n">
         <v>35.43</v>
@@ -1937,7 +1937,7 @@
         <v>105.07</v>
       </c>
       <c r="K7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.015 (auto — vs 1.015 auto)</t>
+          <t>1.026 (auto — vs 1.026 auto)</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.015</t>
+          <t>1.026</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-29 10:11:10</t>
+          <t>2026-05-29 11:35:45</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2522,12 +2522,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.015</t>
+          <t>1.026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.015</t>
+          <t>1.026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
2026-06-01: cancelaciones Darya+Derek, altas Cynthia+Hannah
- HMNKEKCM4M (Darya Kramar jun→jul, 1110.66€): cancelación flexible
- HMAZFDQRF3 (Derek, ya registrada 29/05): confirmada flexible
- HMAY3W3RB8 (Cynthia Laure, jun 22-24, 2n, 206.04€, NRF): nueva
- HMKQFE28R9 (Hannah P., jul 3-6, 3n, 375.27€, NRF): nueva
- baseline 2026-07 actualizado: 3161.65→2537.33, 27n→21n
- T1 auditar_dashboard.py adaptado (Darya ahora cancelada)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -597,41 +597,41 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>83.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>56.48</v>
+        <v>75.06</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>58.94</v>
+        <v>78.67</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>60.25</v>
+        <v>82.2</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -640,237 +640,249 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>P25–P40  (56€–58€)</t>
+          <t>P25–P40  (75€–78€)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>57.06</v>
+        <v>76.53</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>56.94</v>
+        <v>76.23</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>51.25</v>
+        <v>68.61</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Hueco próximo — revisar diariamente</t>
+          <t>Revisar 2026-06-03; sin vender → bajar 5–10%</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>56.48</v>
+        <v>67.55</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>68.08</v>
+        <v>92.89</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="F3" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>84.40000000000001</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>75.06</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="3" t="n">
         <v>78.67</v>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>82.42</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (75€–78€)</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>76.53</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>76.53</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>68.88</v>
-      </c>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-03; sin vender → bajar 5–10%</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="n">
-        <v>67.55</v>
-      </c>
-      <c r="X3" s="2" t="n">
-        <v>93.13</v>
+      <c r="J3" s="3" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (78€–81€)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>80.03</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>72.03</v>
+      </c>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="n"/>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-13; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>75.06</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>92.89</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>86.7</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>75.06</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>78.67</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>82.42</v>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (78€–81€)</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>79.81</v>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>80.09999999999999</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>72.09</v>
-      </c>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-07; sin vender → bajar 5–10%</t>
-        </is>
-      </c>
-      <c r="W4" s="3" t="n">
-        <v>75.06</v>
-      </c>
-      <c r="X4" s="3" t="n">
-        <v>93.13</v>
+      <c r="F4" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>100.41</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>105.09</v>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>P65–P75  (104€–105€)</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>104.67</v>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>94.41</v>
+      </c>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-06; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>118.75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -878,7 +890,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -887,19 +899,19 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>88.90000000000001</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>75.06</v>
+        <v>92.25</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>78.67</v>
+        <v>100.41</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>82.42</v>
+        <v>105.09</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -908,73 +920,73 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (81€–82€)</t>
+          <t>P65–P75  (104€–105€)</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>81.94</v>
+        <v>104.67</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
-        <v>82.05</v>
+        <v>104.8</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>73.84</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>Revisar 2026-05-29; sin vender → bajar 5%</t>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W5" s="4" t="n">
-        <v>75.06</v>
+        <v>92.25</v>
       </c>
       <c r="X5" s="4" t="n">
-        <v>93.13</v>
+        <v>118.75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -983,19 +995,19 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>88.90000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>92.25</v>
+        <v>93.75</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>100.41</v>
+        <v>99</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>105.03</v>
+        <v>105.81</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
@@ -1004,286 +1016,286 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (104€–105€)</t>
+          <t>P65–P75  (102€–106€)</t>
         </is>
       </c>
       <c r="M6" s="4" t="n">
-        <v>104.64</v>
+        <v>103.9</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>buena antelación (↑15%)</t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>104.9</v>
+        <v>104.47</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>94.41</v>
+        <v>94.02</v>
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%).</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-10; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W6" s="4" t="n">
-        <v>92.25</v>
+        <v>93.75</v>
       </c>
       <c r="X6" s="4" t="n">
-        <v>118.68</v>
+        <v>119.57</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>92.25</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>100.41</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>105.03</v>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>P65–P75  (104€–105€)</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>104.64</v>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>104.9</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>94.41</v>
-      </c>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="n">
-        <v>92.25</v>
-      </c>
-      <c r="X7" s="4" t="n">
-        <v>118.68</v>
+      <c r="F7" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>105.81</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (97€–100€)</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>98.86</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>89.11</v>
+      </c>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>119.57</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>77</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>105.81</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–106€)</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>103.9</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>104.85</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>94.36</v>
-      </c>
-      <c r="Q8" s="4" t="n"/>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="X8" s="4" t="n">
-        <v>119.57</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–56€)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>48.36</v>
+      </c>
+      <c r="Q8" s="2" t="n"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>75.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>91</v>
+        <v>133</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>52.2</v>
+        <v>17.8</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>93.75</v>
+        <v>52.08</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>99</v>
+        <v>60.1</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>105.81</v>
+        <v>66.44</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1292,345 +1304,153 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (97€–100€)</t>
+          <t>P45–P60  (57€–61€)</t>
         </is>
       </c>
       <c r="M9" s="3" t="n">
-        <v>98.86</v>
+        <v>59.16</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O9" s="3" t="n">
-        <v>99.31999999999999</v>
+        <v>59.37</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>89.39</v>
-      </c>
-      <c r="Q9" s="3" t="n"/>
+        <v>53.43</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>394.81</v>
+      </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W9" s="3" t="n">
-        <v>93.75</v>
+        <v>52.08</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>119.57</v>
+        <v>75.08</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-23</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>153</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>321.19</v>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>126</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="P10" s="2" t="n">
-        <v>48.69</v>
-      </c>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W10" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X10" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>136</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q11" s="3" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S11" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T11" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U11" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V11" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W11" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X11" s="3" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>52</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>156</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H12" s="3" t="n">
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W10" s="3" t="n">
         <v>43.9</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O12" s="3" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>43.56</v>
-      </c>
-      <c r="Q12" s="3" t="n">
-        <v>321.86</v>
-      </c>
-      <c r="R12" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S12" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U12" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V12" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W12" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X12" s="3" t="n">
+      <c r="X10" s="3" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1922,19 +1742,19 @@
         <v>78.67</v>
       </c>
       <c r="F7" t="n">
-        <v>81.25</v>
+        <v>81.13</v>
       </c>
       <c r="G7" t="n">
-        <v>81.45</v>
+        <v>81.33</v>
       </c>
       <c r="H7" t="n">
-        <v>82.42</v>
+        <v>82.2</v>
       </c>
       <c r="I7" t="n">
         <v>35.43</v>
       </c>
       <c r="J7" t="n">
-        <v>105.07</v>
+        <v>92.43000000000001</v>
       </c>
       <c r="K7" t="n">
         <v>31</v>
@@ -1965,13 +1785,13 @@
         <v>104.25</v>
       </c>
       <c r="H8" t="n">
-        <v>105.03</v>
+        <v>105.09</v>
       </c>
       <c r="I8" t="n">
         <v>81.5</v>
       </c>
       <c r="J8" t="n">
-        <v>116</v>
+        <v>116.77</v>
       </c>
       <c r="K8" t="n">
         <v>28</v>
@@ -2237,7 +2057,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2093,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.026 (auto — vs 1.026 auto)</t>
+          <t>0.996 (auto — vs 0.996 auto)</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2105,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.026</t>
+          <t>0.996</t>
         </is>
       </c>
     </row>
@@ -2502,12 +2322,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-29 11:35:45</t>
+          <t>2026-06-01 08:34:46</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2522,17 +2342,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.026</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.026</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Alta Britta John (HM8T2PNRSC): jul 6-12, 6n, 718.73€ NRF
Cubre el hueco Jul 6-12 dejado por Darya Kramar.
Julio 2026: 27n/31 = 87% ocupacion, 3.256 EUR.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -454,7 +454,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
@@ -622,7 +622,7 @@
         <v>17</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>78.90000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.06</v>
@@ -648,19 +648,19 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76.23</v>
+        <v>76.53</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.61</v>
+        <v>68.88</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -714,7 +714,7 @@
         <v>27</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>75.06</v>
@@ -740,19 +740,19 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O3" s="3" t="n">
-        <v>80.03</v>
+        <v>80.3</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>72.03</v>
+        <v>72.27</v>
       </c>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: ocupación futura alta (↑10%).</t>
+          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S3" s="3" t="n"/>
@@ -781,16 +781,16 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>88.90000000000001</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>92.25</v>
+        <v>93</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>100.41</v>
+        <v>101.5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>105.09</v>
+        <v>105.33</v>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
@@ -824,73 +824,73 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (104€–105€)</t>
+          <t>P65–P75  (105€–105€)</t>
         </is>
       </c>
       <c r="M4" s="4" t="n">
-        <v>104.67</v>
+        <v>105.16</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O4" s="4" t="n">
-        <v>104.9</v>
+        <v>105.65</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>94.41</v>
+        <v>95.09</v>
       </c>
       <c r="Q4" s="4" t="n"/>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="V4" s="4" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-06; sin vender → bajar 5%</t>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W4" s="4" t="n">
-        <v>92.25</v>
+        <v>93</v>
       </c>
       <c r="X4" s="4" t="n">
-        <v>118.75</v>
+        <v>119.02</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -899,19 +899,19 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>75.59999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>92.25</v>
+        <v>93.75</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>100.41</v>
+        <v>99</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>105.09</v>
+        <v>105.81</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -920,382 +920,384 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (104€–105€)</t>
+          <t>P65–P75  (102€–106€)</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>104.67</v>
+        <v>103.9</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
-        <v>104.8</v>
+        <v>104.85</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>94.31999999999999</v>
+        <v>94.36</v>
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W5" s="4" t="n">
-        <v>92.25</v>
+        <v>93.75</v>
       </c>
       <c r="X5" s="4" t="n">
-        <v>118.75</v>
+        <v>119.57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>74</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="H6" s="4" t="n">
+      <c r="F6" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>93.75</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="3" t="n">
         <v>105.81</v>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–106€)</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>103.9</v>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%)</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>104.47</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>94.02</v>
-      </c>
-      <c r="Q6" s="4" t="n"/>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%).</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="n">
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (97€–100€)</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>98.86</v>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>89.39</v>
+      </c>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="n">
         <v>93.75</v>
       </c>
-      <c r="X6" s="4" t="n">
+      <c r="X6" s="3" t="n">
         <v>119.57</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>88</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>99</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>105.81</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–56€)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>48.69</v>
+      </c>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>75.08</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (97€–100€)</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>98.86</v>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>99.01000000000001</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>89.11</v>
-      </c>
-      <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>119.57</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>123</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H8" s="2" t="n">
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>397.67</v>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="n">
         <v>52.08</v>
       </c>
-      <c r="I8" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>53.73</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>48.36</v>
-      </c>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X8" s="2" t="n">
+      <c r="X8" s="3" t="n">
         <v>75.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-12-23</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>baja</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>17.8</v>
+        <v>11.1</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>52.08</v>
+        <v>43.9</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>60.1</v>
+        <v>47.75</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>66.44</v>
+        <v>50</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1304,153 +1306,55 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (57€–61€)</t>
+          <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
       <c r="M9" s="3" t="n">
-        <v>59.16</v>
+        <v>48.17</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O9" s="3" t="n">
-        <v>59.37</v>
+        <v>48.4</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>53.43</v>
+        <v>43.56</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>394.81</v>
+        <v>321.86</v>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W9" s="3" t="n">
-        <v>52.08</v>
+        <v>43.9</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>52</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>153</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="I10" s="3" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>43.47</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>321.19</v>
-      </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V10" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W10" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X10" s="3" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1472,9 +1376,9 @@
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -1767,34 +1671,34 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>92.25</v>
+        <v>93</v>
       </c>
       <c r="C8" t="n">
-        <v>98.40000000000001</v>
+        <v>98.76000000000001</v>
       </c>
       <c r="D8" t="n">
         <v>99.33</v>
       </c>
       <c r="E8" t="n">
-        <v>100.41</v>
+        <v>101.5</v>
       </c>
       <c r="F8" t="n">
-        <v>103.2</v>
+        <v>103.3</v>
       </c>
       <c r="G8" t="n">
-        <v>104.25</v>
+        <v>105</v>
       </c>
       <c r="H8" t="n">
-        <v>105.09</v>
+        <v>105.33</v>
       </c>
       <c r="I8" t="n">
         <v>81.5</v>
       </c>
       <c r="J8" t="n">
-        <v>116.77</v>
+        <v>121.99</v>
       </c>
       <c r="K8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -2093,7 +1997,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.996 (auto — vs 0.996 auto)</t>
+          <t>1.037 (auto — vs 1.037 auto)</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2009,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.996</t>
+          <t>1.037</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2226,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-01 08:34:46</t>
+          <t>2026-06-01 09:27:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2342,17 +2246,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.996</t>
+          <t>1.037</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.996</t>
+          <t>1.037</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva: Rachel Pons Gual De Torrella (HM4M9WT2QE) — Jul 2, 1n, 155.16EUR
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -454,7 +454,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
@@ -467,7 +467,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="51" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>85.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.06</v>
@@ -664,11 +664,7 @@
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>2026-06-11</t>
@@ -676,7 +672,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-03; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-06-11; sin vender → precio Ocupación</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -694,11 +690,11 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -711,7 +707,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>91.09999999999999</v>
@@ -740,19 +736,19 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O3" s="3" t="n">
-        <v>80.3</v>
+        <v>80.03</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>72.27</v>
+        <v>72.03</v>
       </c>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + ocupación futura alta (↑10%).</t>
+          <t>Equilibrio (temporada alta + antelación justa). Precio de mercado balanceado. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S3" s="3" t="n"/>
@@ -803,19 +799,19 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>75.59999999999999</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>93</v>
+        <v>93.25</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>101.5</v>
+        <v>100.41</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>105.33</v>
+        <v>105.25</v>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
@@ -828,7 +824,7 @@
         </is>
       </c>
       <c r="M4" s="4" t="n">
-        <v>105.16</v>
+        <v>105</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
@@ -836,10 +832,10 @@
         </is>
       </c>
       <c r="O4" s="4" t="n">
-        <v>105.65</v>
+        <v>105.4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>95.09</v>
+        <v>94.86</v>
       </c>
       <c r="Q4" s="4" t="n"/>
       <c r="R4" s="4" t="inlineStr">
@@ -868,10 +864,10 @@
         </is>
       </c>
       <c r="W4" s="4" t="n">
-        <v>93</v>
+        <v>93.25</v>
       </c>
       <c r="X4" s="4" t="n">
-        <v>119.02</v>
+        <v>118.93</v>
       </c>
     </row>
     <row r="5">
@@ -899,7 +895,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>63.3</v>
@@ -995,7 +991,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>52.2</v>
@@ -1091,7 +1087,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>26.7</v>
@@ -1187,7 +1183,7 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>17.8</v>
@@ -1285,7 +1281,7 @@
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>11.1</v>
@@ -1376,9 +1372,9 @@
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -1671,25 +1667,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>93</v>
+        <v>93.25</v>
       </c>
       <c r="C8" t="n">
-        <v>98.76000000000001</v>
+        <v>98.17</v>
       </c>
       <c r="D8" t="n">
         <v>99.33</v>
       </c>
       <c r="E8" t="n">
-        <v>101.5</v>
+        <v>100.41</v>
       </c>
       <c r="F8" t="n">
-        <v>103.3</v>
+        <v>103.23</v>
       </c>
       <c r="G8" t="n">
-        <v>105</v>
+        <v>104.75</v>
       </c>
       <c r="H8" t="n">
-        <v>105.33</v>
+        <v>105.25</v>
       </c>
       <c r="I8" t="n">
         <v>81.5</v>
@@ -1698,7 +1694,7 @@
         <v>121.99</v>
       </c>
       <c r="K8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -1961,7 +1957,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1993,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.037 (auto — vs 1.037 auto)</t>
+          <t>1.027 (auto — vs 1.027 auto)</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2005,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.037</t>
+          <t>1.027</t>
         </is>
       </c>
     </row>
@@ -2226,12 +2222,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-01 09:27:25</t>
+          <t>2026-06-08 15:17:39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2246,12 +2242,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.037</t>
+          <t>1.027</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.037</t>
+          <t>1.027</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva: Anne Ooms (HMF95F5PJM) — Jun 29, 3n cross-month, 346.64EUR
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -622,16 +622,16 @@
         <v>10</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>86.7</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>75.06</v>
+        <v>75.08</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>78.67</v>
+        <v>79</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>82.2</v>
+        <v>82.38</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>76.53</v>
+        <v>76.61</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -652,10 +652,10 @@
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76.53</v>
+        <v>76.61</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.88</v>
+        <v>68.95</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
@@ -676,217 +676,213 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>67.55</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>92.89</v>
+        <v>93.09</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>75.08</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>82.38</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (75€–78€)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>76.61</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>76.61</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>68.95</v>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-13; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>67.56999999999999</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>93.09</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" s="3" t="n">
+      <c r="F4" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>91.09999999999999</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>75.06</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>78.67</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>82.2</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="H4" s="3" t="n">
+        <v>93.25</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>100.41</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (78€–81€)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>80.03</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>72.03</v>
-      </c>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta + antelación justa). Precio de mercado balanceado. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-13; sin vender → bajar 5–10%</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>75.06</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>92.89</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>100.41</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>105.25</v>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>P65–P75  (105€–105€)</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (99€–103€)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>101.28</v>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>105.4</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>94.86</v>
-      </c>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="X4" s="4" t="n">
+      <c r="O4" s="3" t="n">
+        <v>101.67</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-16; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="X4" s="3" t="n">
         <v>118.93</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -895,19 +891,19 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>63.3</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>93.75</v>
+        <v>93.25</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>99</v>
+        <v>100.41</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>105.81</v>
+        <v>105.25</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -916,441 +912,537 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (102€–106€)</t>
+          <t>P65–P75  (105€–105€)</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>103.9</v>
+        <v>105</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
-        <v>104.85</v>
+        <v>105.4</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>94.36</v>
+        <v>94.86</v>
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="inlineStr">
         <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>93.25</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>118.93</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>105.81</v>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–106€)</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>94.36</v>
+      </c>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
           <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W5" s="4" t="n">
+      <c r="W6" s="4" t="n">
         <v>93.75</v>
       </c>
-      <c r="X5" s="4" t="n">
+      <c r="X6" s="4" t="n">
         <v>119.57</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F7" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G7" s="3" t="n">
         <v>52.2</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H7" s="3" t="n">
         <v>93.75</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I7" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>105.81</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (97€–100€)</t>
         </is>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="M7" s="3" t="n">
         <v>98.86</v>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
-      <c r="O6" s="3" t="n">
+      <c r="O7" s="3" t="n">
         <v>99.31999999999999</v>
       </c>
-      <c r="P6" s="3" t="n">
+      <c r="P7" s="3" t="n">
         <v>89.39</v>
       </c>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="U6" s="3" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="V6" s="3" t="inlineStr">
+      <c r="V7" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W6" s="3" t="n">
+      <c r="W7" s="3" t="n">
         <v>93.75</v>
       </c>
-      <c r="X6" s="3" t="n">
+      <c r="X7" s="3" t="n">
         <v>119.57</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>116</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>26.7</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>60.1</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>66.44</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>53.92</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O8" s="2" t="n">
         <v>54.1</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P8" s="2" t="n">
         <v>48.69</v>
       </c>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="n"/>
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W7" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="X7" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>126</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U8" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V8" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X8" s="3" t="n">
+      <c r="X8" s="2" t="n">
         <v>75.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>397.67</v>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>75.08</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C10" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F10" s="3" t="n">
         <v>146</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G10" s="3" t="n">
         <v>11.1</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H10" s="3" t="n">
         <v>43.9</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I10" s="3" t="n">
         <v>47.75</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="J10" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="M10" s="3" t="n">
         <v>48.17</v>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O9" s="3" t="n">
+      <c r="O10" s="3" t="n">
         <v>48.4</v>
       </c>
-      <c r="P9" s="3" t="n">
+      <c r="P10" s="3" t="n">
         <v>43.56</v>
       </c>
-      <c r="Q9" s="3" t="n">
+      <c r="Q10" s="3" t="n">
         <v>321.86</v>
       </c>
-      <c r="R9" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S9" s="3" t="inlineStr">
+      <c r="S10" s="3" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="T9" s="3" t="inlineStr">
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="U9" s="3" t="inlineStr">
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="V9" s="3" t="inlineStr">
+      <c r="V10" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W9" s="3" t="n">
+      <c r="W10" s="3" t="n">
         <v>43.9</v>
       </c>
-      <c r="X9" s="3" t="n">
+      <c r="X10" s="3" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1630,34 +1722,34 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>75.06</v>
+        <v>75.08</v>
       </c>
       <c r="C7" t="n">
-        <v>78</v>
+        <v>78.13</v>
       </c>
       <c r="D7" t="n">
-        <v>78.38</v>
+        <v>78.42</v>
       </c>
       <c r="E7" t="n">
-        <v>78.67</v>
+        <v>79</v>
       </c>
       <c r="F7" t="n">
-        <v>81.13</v>
+        <v>81.2</v>
       </c>
       <c r="G7" t="n">
-        <v>81.33</v>
+        <v>81.42</v>
       </c>
       <c r="H7" t="n">
-        <v>82.2</v>
+        <v>82.38</v>
       </c>
       <c r="I7" t="n">
         <v>35.43</v>
       </c>
       <c r="J7" t="n">
-        <v>92.43000000000001</v>
+        <v>95.55</v>
       </c>
       <c r="K7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
@@ -1993,7 +2085,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.027 (auto — vs 1.027 auto)</t>
+          <t>1.038 (auto — vs 1.038 auto)</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2097,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.027</t>
+          <t>1.038</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2314,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-08 15:17:39</t>
+          <t>2026-06-08 15:26:57</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2242,17 +2334,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.027</t>
+          <t>1.038</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.027</t>
+          <t>1.038</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Fix: checkin continuacion Anne Ooms julio — elimina hueco falso Jul 1-2
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -51,12 +51,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E8DAEF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8DAEF"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
         <v>10</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>88.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.08</v>
@@ -710,7 +710,7 @@
         <v>20</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>90</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>75.08</v>
@@ -777,16 +777,16 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>91.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>93.25</v>
@@ -815,16 +815,16 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio</t>
+          <t>Rentabilidad</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (99€–103€)</t>
+          <t>P65–P75  (105€–105€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>101.28</v>
+        <v>105</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
@@ -832,149 +832,153 @@
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>101.67</v>
+        <v>105.4</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>91.5</v>
+        <v>94.86</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="n"/>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-16; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>83.92</v>
+        <v>93.25</v>
       </c>
       <c r="X4" s="3" t="n">
         <v>118.93</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>105.81</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–106€)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>94.36</v>
+      </c>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>100.41</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>105.25</v>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>P65–P75  (105€–105€)</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="n">
-        <v>105.4</v>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>94.86</v>
-      </c>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="T5" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W5" s="4" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>118.93</v>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>119.57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -987,10 +991,10 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>63.3</v>
+        <v>52.2</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>93.75</v>
@@ -1003,52 +1007,52 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad</t>
+          <t>Equilibrio</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>P65–P75  (102€–106€)</t>
+          <t>P45–P60  (97€–100€)</t>
         </is>
       </c>
       <c r="M6" s="4" t="n">
-        <v>103.9</v>
+        <v>98.86</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>104.85</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>94.36</v>
+        <v>89.39</v>
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W6" s="4" t="n">
@@ -1059,390 +1063,294 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>81</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>99</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>105.81</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–56€)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>48.69</v>
+      </c>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>75.08</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (97€–100€)</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>98.86</v>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>99.31999999999999</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>89.39</v>
-      </c>
-      <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>119.57</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>397.67</v>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>75.08</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-23</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>43.56</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>321.86</v>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>116</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>48.69</v>
-      </c>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>126</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q9" s="3" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U9" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V9" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W9" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X9" s="3" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>52</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>146</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H10" s="3" t="n">
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n">
         <v>43.9</v>
       </c>
-      <c r="I10" s="3" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>43.56</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>321.86</v>
-      </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U10" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V10" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W10" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X10" s="3" t="n">
+      <c r="X9" s="4" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -2314,7 +2222,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-08 15:26:57</t>
+          <t>2026-06-08 15:35:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2344,7 +2252,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Cancelacion HMHXK9AFY5 Renuka Prabhakar (ago 9-14, 530.04EUR, flexible)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>90</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.08</v>
@@ -648,31 +648,27 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76.61</v>
+        <v>76</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.95</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
+      <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-11; sin vender → precio Ocupación</t>
+          <t>Hueco próximo — revisar diariamente</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -707,10 +703,10 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>91.09999999999999</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>75.08</v>
@@ -736,27 +732,23 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>76.61</v>
+        <v>76.3</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>68.95</v>
+        <v>68.67</v>
       </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
+      <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -764,7 +756,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-13; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-06-21; sin vender → precio Ocupación</t>
         </is>
       </c>
       <c r="W3" s="2" t="n">
@@ -799,10 +791,10 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>70</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>93.25</v>
@@ -828,19 +820,19 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>105.4</v>
+        <v>105.3</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>94.86</v>
+        <v>94.77</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
@@ -873,7 +865,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -882,7 +874,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -895,19 +887,19 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>63.3</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>93.75</v>
+        <v>93.62</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>99</v>
+        <v>99.12</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>105.81</v>
+        <v>106.2</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -920,50 +912,52 @@
         </is>
       </c>
       <c r="M5" s="3" t="n">
-        <v>103.9</v>
+        <v>104.1</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%)</t>
+          <t>tensión +4% sobre P75</t>
         </is>
       </c>
       <c r="O5" s="3" t="n">
-        <v>104.85</v>
+        <v>110.45</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>94.36</v>
-      </c>
-      <c r="Q5" s="3" t="n"/>
+        <v>99.41</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>734.49</v>
+      </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%).</t>
+          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: tensión +4% sobre P75.</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-15; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-10; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W5" s="3" t="n">
-        <v>93.75</v>
+        <v>93.62</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>119.57</v>
+        <v>120.01</v>
       </c>
     </row>
     <row r="6">
@@ -991,19 +985,19 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>52.2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>93.75</v>
+        <v>93.62</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>99</v>
+        <v>99.12</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>105.81</v>
+        <v>106.2</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
@@ -1012,27 +1006,27 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>P45–P60  (97€–100€)</t>
+          <t>P45–P60  (98€–101€)</t>
         </is>
       </c>
       <c r="M6" s="4" t="n">
-        <v>98.86</v>
+        <v>99.61</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>99.31999999999999</v>
+        <v>99.75</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>89.39</v>
+        <v>89.78</v>
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
@@ -1056,10 +1050,10 @@
         </is>
       </c>
       <c r="W6" s="4" t="n">
-        <v>93.75</v>
+        <v>93.62</v>
       </c>
       <c r="X6" s="4" t="n">
-        <v>119.57</v>
+        <v>120.01</v>
       </c>
     </row>
     <row r="7">
@@ -1087,7 +1081,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>26.7</v>
@@ -1116,19 +1110,19 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
-        <v>54.1</v>
+        <v>53.73</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>48.69</v>
+        <v>48.36</v>
       </c>
       <c r="Q7" s="2" t="n"/>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -1183,7 +1177,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>17.8</v>
@@ -1212,21 +1206,21 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O8" s="4" t="n">
-        <v>59.8</v>
+        <v>59.37</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>53.82</v>
+        <v>53.43</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>397.67</v>
+        <v>394.81</v>
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
@@ -1281,7 +1275,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>11.1</v>
@@ -1310,21 +1304,21 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O9" s="4" t="n">
-        <v>48.4</v>
+        <v>48.3</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>43.56</v>
+        <v>43.47</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>321.86</v>
+        <v>321.19</v>
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr">
@@ -1704,25 +1698,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93.75</v>
+        <v>93.62</v>
       </c>
       <c r="C9" t="n">
-        <v>96.72</v>
+        <v>96.86</v>
       </c>
       <c r="D9" t="n">
-        <v>97.34</v>
+        <v>98.20999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>99</v>
+        <v>99.12</v>
       </c>
       <c r="F9" t="n">
-        <v>100.38</v>
+        <v>101.01</v>
       </c>
       <c r="G9" t="n">
         <v>102</v>
       </c>
       <c r="H9" t="n">
-        <v>105.81</v>
+        <v>106.2</v>
       </c>
       <c r="I9" t="n">
         <v>73</v>
@@ -1731,7 +1725,7 @@
         <v>120</v>
       </c>
       <c r="K9" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
@@ -1957,7 +1951,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1987,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.038 (auto — vs 1.038 auto)</t>
+          <t>1.012 (auto — vs 1.012 auto)</t>
         </is>
       </c>
     </row>
@@ -2005,7 +1999,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>1.012</t>
         </is>
       </c>
     </row>
@@ -2222,12 +2216,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-08 15:35:17</t>
+          <t>2026-06-15 09:38:01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2242,12 +2236,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>1.012</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>1.012</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva HMX25YHD58 Vera francesa (ago 12-17, 5n, 756.50EUR, flexible)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>84.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.08</v>
@@ -648,19 +648,19 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76</v>
+        <v>76.3</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>68.67</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -706,7 +706,7 @@
         <v>13</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>85.59999999999999</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>75.08</v>
@@ -732,19 +732,19 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>76.3</v>
+        <v>76.61</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>68.67</v>
+        <v>68.95</v>
       </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
@@ -794,7 +794,7 @@
         <v>43</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>70</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>93.25</v>
@@ -820,19 +820,19 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>105.3</v>
+        <v>105.4</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>94.77</v>
+        <v>94.86</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
@@ -870,11 +870,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -890,461 +890,555 @@
         <v>55</v>
       </c>
       <c r="G5" s="3" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–107€)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>104.58</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>pickup fuerte (↑10%) + hueco corto (↓5%) + tensión +4% sobre P75</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>111.33</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco corto (↓5%) + tensión +4% sobre P75.</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-10; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>120.97</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>63.3</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>93.62</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>99.12</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>106.2</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="H6" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Rentabilidad</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–106€)</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>104.1</v>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>tensión +4% sobre P75</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>110.45</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>99.41</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>734.49</v>
-      </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: tensión +4% sobre P75.</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="U5" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–107€)</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>104.58</v>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + tensión +4% sobre P75</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>111.33</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + tensión +4% sobre P75.</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="V5" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-10; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W5" s="3" t="n">
-        <v>93.62</v>
-      </c>
-      <c r="X5" s="3" t="n">
-        <v>120.01</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>84.38</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>120.97</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F7" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G7" s="3" t="n">
         <v>52.2</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>93.62</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>99.12</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>106.2</v>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (98€–101€)</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>99.61</v>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>99.75</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>89.78</v>
-      </c>
-      <c r="Q6" s="4" t="n"/>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="H7" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>P65–P75  (102€–107€)</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>104.58</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>105.32</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>94.79000000000001</v>
+      </c>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
+      <c r="V7" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W6" s="4" t="n">
-        <v>93.62</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>120.01</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="W7" s="3" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>120.97</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>26.7</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>60.1</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>66.44</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>53.92</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>53.73</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>48.36</v>
-      </c>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>48.69</v>
+      </c>
+      <c r="Q8" s="2" t="n"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W7" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="X7" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>119</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>59.37</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>53.43</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>394.81</v>
-      </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X8" s="4" t="n">
+      <c r="X8" s="2" t="n">
         <v>75.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>397.67</v>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>75.08</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C10" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>139</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>11.1</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>43.9</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>47.75</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>48.17</v>
       </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>43.47</v>
-      </c>
-      <c r="Q9" s="4" t="n">
-        <v>321.19</v>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>43.56</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>321.86</v>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
+      <c r="T10" s="4" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr">
+      <c r="U10" s="4" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
+      <c r="V10" s="4" t="inlineStr">
         <is>
           <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W9" s="4" t="n">
+      <c r="W10" s="4" t="n">
         <v>43.9</v>
       </c>
-      <c r="X9" s="4" t="n">
+      <c r="X10" s="4" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1698,34 +1792,34 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93.62</v>
+        <v>93.75</v>
       </c>
       <c r="C9" t="n">
         <v>96.86</v>
       </c>
       <c r="D9" t="n">
-        <v>98.20999999999999</v>
+        <v>98.62</v>
       </c>
       <c r="E9" t="n">
-        <v>99.12</v>
+        <v>99.25</v>
       </c>
       <c r="F9" t="n">
-        <v>101.01</v>
+        <v>101.6</v>
       </c>
       <c r="G9" t="n">
-        <v>102</v>
+        <v>102.12</v>
       </c>
       <c r="H9" t="n">
-        <v>106.2</v>
+        <v>107.05</v>
       </c>
       <c r="I9" t="n">
         <v>73</v>
       </c>
       <c r="J9" t="n">
-        <v>120</v>
+        <v>139.3</v>
       </c>
       <c r="K9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -1987,7 +2081,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.012 (auto — vs 1.012 auto)</t>
+          <t>1.051 (auto — vs 1.051 auto)</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2093,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.012</t>
+          <t>1.051</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2310,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-15 09:38:01</t>
+          <t>2026-06-15 09:48:39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2236,17 +2330,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.012</t>
+          <t>1.051</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.012</t>
+          <t>1.051</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
feat: nueva reserva Maria Prachapchuk (HMNH4CEJYJ) ago 9-12 NRF 471.54EUR
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="51" customWidth="1" min="22" max="22"/>
+    <col width="43" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -597,12 +597,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>90</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>75.08</v>
@@ -648,19 +648,19 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>antelación muy baja (↓20%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76.3</v>
+        <v>76.61</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.67</v>
+        <v>68.95</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -679,110 +679,118 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>93.25</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>100.41</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>P65–P75  (105€–105€)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>94.95</v>
+      </c>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>75.08</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>82.38</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (75€–78€)</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>76.61</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>76.61</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>68.95</v>
-      </c>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-21; sin vender → precio Ocupación</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="n">
-        <v>67.56999999999999</v>
-      </c>
-      <c r="X3" s="2" t="n">
-        <v>93.09</v>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>93.25</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>118.93</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -791,19 +799,19 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>93.25</v>
+        <v>93.88</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>100.41</v>
+        <v>99.5</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>105.25</v>
+        <v>107.5</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -812,69 +820,69 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P65–P75  (105€–105€)</t>
+          <t>P65–P75  (103€–108€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>105</v>
+        <v>105.19</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + tensión +4% sobre P75</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>105.4</v>
+        <v>111.8</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>94.86</v>
+        <v>100.62</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + tensión +4% sobre P75.</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>93.25</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>118.93</v>
+        <v>121.47</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -887,19 +895,19 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>68.90000000000001</v>
+        <v>52.2</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>93.75</v>
+        <v>93.88</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>99.25</v>
+        <v>99.5</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>107.05</v>
+        <v>107.5</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -908,537 +916,345 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>P65–P75  (102€–107€)</t>
+          <t>P65–P75  (103€–108€)</t>
         </is>
       </c>
       <c r="M5" s="3" t="n">
-        <v>104.58</v>
+        <v>105.19</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco corto (↓5%) + tensión +4% sobre P75</t>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O5" s="3" t="n">
-        <v>111.33</v>
+        <v>106.34</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>100.2</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="Q5" s="3" t="n"/>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup fuerte (↑10%) + hueco corto (↓5%) + tensión +4% sobre P75.</t>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-10; sin vender → bajar 5%</t>
+          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W5" s="3" t="n">
-        <v>93.75</v>
+        <v>93.88</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>120.97</v>
+        <v>121.47</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>99.25</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>107.05</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–107€)</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>104.58</v>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + tensión +4% sobre P75</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>111.33</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + tensión +4% sobre P75.</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="U6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="3" t="n">
-        <v>84.38</v>
-      </c>
-      <c r="X6" s="3" t="n">
-        <v>120.97</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–56€)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>54.47</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>75.08</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>74</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>99.25</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>107.05</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (102€–107€)</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>104.58</v>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>105.32</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>94.79000000000001</v>
-      </c>
-      <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>120.97</v>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>60.23</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>400.53</v>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>75.08</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-23</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>132</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>322.52</v>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>48.69</v>
-      </c>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>119</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q9" s="4" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X9" s="4" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>139</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H10" s="4" t="n">
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>43.9</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>43.56</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>321.86</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S10" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X10" s="4" t="n">
+      <c r="X8" s="4" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1792,34 +1608,34 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93.75</v>
+        <v>93.88</v>
       </c>
       <c r="C9" t="n">
         <v>96.86</v>
       </c>
       <c r="D9" t="n">
-        <v>98.62</v>
+        <v>98.86</v>
       </c>
       <c r="E9" t="n">
-        <v>99.25</v>
+        <v>99.5</v>
       </c>
       <c r="F9" t="n">
-        <v>101.6</v>
+        <v>102</v>
       </c>
       <c r="G9" t="n">
-        <v>102.12</v>
+        <v>102.88</v>
       </c>
       <c r="H9" t="n">
-        <v>107.05</v>
+        <v>107.5</v>
       </c>
       <c r="I9" t="n">
         <v>73</v>
       </c>
       <c r="J9" t="n">
-        <v>139.3</v>
+        <v>152.42</v>
       </c>
       <c r="K9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
@@ -2045,7 +1861,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2081,7 +1897,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.051 (auto — vs 1.051 auto)</t>
+          <t>1.076 (auto — vs 1.076 auto)</t>
         </is>
       </c>
     </row>
@@ -2093,7 +1909,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.051</t>
+          <t>1.076</t>
         </is>
       </c>
     </row>
@@ -2310,12 +2126,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-15 09:55:45</t>
+          <t>2026-06-22 08:40:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2330,17 +2146,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.051</t>
+          <t>1.076</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.051</t>
+          <t>1.076</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva HM8Z8HTK9D (Nadezhda, 28-30 jul) + reviews Rachel 5/5 y Wilmer 5/5
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -46,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE9D9"/>
+        <fgColor rgb="00E8DAEF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8DAEF"/>
+        <fgColor rgb="00FDE9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -454,8 +454,8 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
@@ -597,12 +597,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -610,7 +610,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -619,642 +619,462 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>94.40000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>75.08</v>
+        <v>93.88</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>79</v>
+        <v>99.5</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>82.38</v>
+        <v>107.5</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación</t>
+          <t>Rentabilidad</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>P25–P40  (75€–78€)</t>
+          <t>P65–P75  (103€–108€)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>76.61</v>
+        <v>105.19</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>76.61</v>
+        <v>105.88</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>68.95</v>
+        <v>95.29000000000001</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Hueco próximo — revisar diariamente</t>
+          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>67.56999999999999</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>93.09</v>
+        <v>121.47</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>78.90000000000001</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>100.41</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>105.25</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>93.88</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Rentabilidad</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (105€–105€)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>105</v>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>105.5</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>94.95</v>
-      </c>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-06-28; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>93.25</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>118.93</v>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>P65–P75  (103€–108€)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>105.19</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>105.88</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>95.29000000000001</v>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>93.88</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>121.47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>63.3</v>
+        <v>26.7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>93.88</v>
+        <v>52.08</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>99.5</v>
+        <v>60.1</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>107.5</v>
+        <v>66.44</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad</t>
+          <t>Ocupación</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P65–P75  (103€–108€)</t>
+          <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>105.19</v>
+        <v>53.92</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + tensión +4% sobre P75</t>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>111.8</v>
+        <v>54.47</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>100.62</v>
+        <v>49.02</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + tensión +4% sobre P75.</t>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>84.48999999999999</v>
+        <v>52.08</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>121.47</v>
+        <v>75.08</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>93.88</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>107.5</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>P65–P75  (103€–108€)</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>105.19</v>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>106.34</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>95.70999999999999</v>
-      </c>
-      <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V5" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W5" s="3" t="n">
-        <v>93.88</v>
-      </c>
-      <c r="X5" s="3" t="n">
-        <v>121.47</v>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>66.44</v>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (57€–61€)</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>60.23</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>400.53</v>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>75.08</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-23</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>322.52</v>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>102</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>54.47</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X6" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>112</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>60.23</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>54.21</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>400.53</v>
-      </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S7" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X7" s="4" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>132</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H8" s="4" t="n">
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="n">
         <v>43.9</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>322.52</v>
-      </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X8" s="4" t="n">
+      <c r="X6" s="4" t="n">
         <v>56.5</v>
       </c>
     </row>
@@ -1276,7 +1096,7 @@
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
@@ -1571,34 +1391,34 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>93.25</v>
+        <v>93.5</v>
       </c>
       <c r="C8" t="n">
-        <v>98.17</v>
+        <v>98.62</v>
       </c>
       <c r="D8" t="n">
         <v>99.33</v>
       </c>
       <c r="E8" t="n">
-        <v>100.41</v>
+        <v>101.5</v>
       </c>
       <c r="F8" t="n">
-        <v>103.23</v>
+        <v>103.33</v>
       </c>
       <c r="G8" t="n">
-        <v>104.75</v>
+        <v>105</v>
       </c>
       <c r="H8" t="n">
-        <v>105.25</v>
+        <v>107.44</v>
       </c>
       <c r="I8" t="n">
         <v>81.5</v>
       </c>
       <c r="J8" t="n">
-        <v>121.99</v>
+        <v>131.9</v>
       </c>
       <c r="K8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -1861,7 +1681,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1717,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.076 (auto — vs 1.076 auto)</t>
+          <t>1.075 (auto — vs 1.075 auto)</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1729,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.076</t>
+          <t>1.075</t>
         </is>
       </c>
     </row>
@@ -2126,12 +1946,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-22 08:40:03</t>
+          <t>2026-07-07 12:41:06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2146,17 +1966,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.076</t>
+          <t>1.075</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.076</t>
+          <t>1.075</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Añade reservas Tomas Pareto y Margarita Trejos, reviews Xepe y Susan
Nuevas reservas HMJJH3HD93 (may 2027) y HMZ5KBRMKK (dic 2026); baseline
de diciembre 2026 actualizado tras el nuevo ingreso. Reviews de Xepe
De Lucas y Susan Schimmeyer añadidas a reviews.json.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -32,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -42,11 +42,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8DAEF"/>
       </patternFill>
     </fill>
     <fill>
@@ -72,12 +67,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,21 +437,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
@@ -467,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="43" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -619,7 +613,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>63.3</v>
@@ -635,39 +629,35 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Rentabilidad</t>
+          <t>Ocupación</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>P65–P75  (103€–108€)</t>
+          <t>P25–P40  (94€–97€)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>105.19</v>
+        <v>95.37</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>105.88</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>95.29000000000001</v>
+        <v>85.56</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación + ocupación futura alta). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>2026-08-02</t>
@@ -680,7 +670,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-07-18; sin vender → bajar 5%</t>
+          <t>Revisar 2026-08-02; sin vender → bajar 5–10%</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -691,391 +681,489 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="F3" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>52.2</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>93.88</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="3" t="n">
         <v>99.5</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="3" t="n">
         <v>107.5</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>P65–P75  (103€–108€)</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>105.19</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>pickup muy fuerte (↑20%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>105.88</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>95.29000000000001</v>
-      </c>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Rentabilidad (temporada alta + pickup fuerte + suficiente antelación). Objetivo: defender ADR sin descuento innecesario. Ajustes en zona: pickup muy fuerte (↑20%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (99€–102€)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>100.43</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>100.59</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>90.53</v>
+      </c>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr">
+      <c r="V3" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W3" s="2" t="n">
+      <c r="W3" s="3" t="n">
         <v>93.88</v>
       </c>
-      <c r="X3" s="2" t="n">
+      <c r="X3" s="3" t="n">
         <v>121.47</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>87</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H4" s="3" t="n">
+      <c r="F4" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="2" t="n">
         <v>60.1</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>66.44</v>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="M4" s="2" t="n">
         <v>53.92</v>
       </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="n">
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="n">
         <v>54.47</v>
       </c>
-      <c r="P4" s="3" t="n">
+      <c r="P4" s="2" t="n">
         <v>49.02</v>
       </c>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="W4" s="2" t="n">
         <v>52.08</v>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="X4" s="2" t="n">
         <v>75.08</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>97</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H5" s="4" t="n">
+      <c r="F5" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>52.08</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="3" t="n">
         <v>60.1</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="3" t="n">
         <v>66.44</v>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (57€–61€)</t>
         </is>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M5" s="3" t="n">
         <v>59.16</v>
       </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="n">
-        <v>60.23</v>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>54.21</v>
-      </c>
-      <c r="Q5" s="4" t="n">
-        <v>400.53</v>
-      </c>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>397.67</v>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
+      <c r="V5" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W5" s="4" t="n">
+      <c r="W5" s="3" t="n">
         <v>52.08</v>
       </c>
-      <c r="X5" s="4" t="n">
+      <c r="X5" s="3" t="n">
         <v>75.08</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>43.56</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>321.86</v>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="C7" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Diciembre (1-19)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>117</v>
-      </c>
-      <c r="G6" s="4" t="n">
+      <c r="F7" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="G7" s="3" t="n">
         <v>11.1</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="H7" s="3" t="n">
+        <v>42.03</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>322.52</v>
-      </c>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup muy fuerte (↑20%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>56.5</v>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (43€–45€)</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>43.83</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>44.07</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>39.66</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>293.07</v>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>42.03</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>52.74</v>
       </c>
     </row>
   </sheetData>
@@ -1576,25 +1664,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>41.71</v>
+        <v>42.03</v>
       </c>
       <c r="C13" t="n">
         <v>43</v>
       </c>
       <c r="D13" t="n">
-        <v>43</v>
+        <v>43.05</v>
       </c>
       <c r="E13" t="n">
-        <v>43</v>
+        <v>43.45</v>
       </c>
       <c r="F13" t="n">
-        <v>43.72</v>
+        <v>44.62</v>
       </c>
       <c r="G13" t="n">
-        <v>44.26</v>
+        <v>45.43</v>
       </c>
       <c r="H13" t="n">
-        <v>45.7</v>
+        <v>46.67</v>
       </c>
       <c r="I13" t="n">
         <v>38.33</v>
@@ -1603,7 +1691,7 @@
         <v>51.5</v>
       </c>
       <c r="K13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1681,7 +1769,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1805,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.075 (auto — vs 1.075 auto)</t>
+          <t>1.021 (auto — vs 1.021 auto)</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1817,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.075</t>
+          <t>1.021</t>
         </is>
       </c>
     </row>
@@ -1946,12 +2034,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-07 12:41:06</t>
+          <t>2026-07-28 10:45:22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1966,17 +2054,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.075</t>
+          <t>1.021</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.075</t>
+          <t>1.021</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva Alexzandra Echevarria (HMSM4KHR9E, jun 2027) + cancelación Hermann (HMZMSSNHFH)
La reserva de Hermann (08-25 jun 2027) se solapaba con la nueva de
Alexzandra (16-21 jun 2027); Hermann canceló sin penalización. Baseline
2027-06 actualizado tras el cambio de ingreso.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>63.3</v>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>52.2</v>
@@ -738,10 +738,10 @@
         </is>
       </c>
       <c r="O3" s="3" t="n">
-        <v>100.59</v>
+        <v>100.43</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>90.53</v>
+        <v>90.39</v>
       </c>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="inlineStr">
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>31.1</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>22.2</v>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>15.6</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>11.1</v>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2034,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-28 10:45:22</t>
+          <t>2026-07-29 14:07:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva: Bernhard Bugenhagen (HM92X8PQ8T)
13-19 oct 2026, 6 noches, 477.72EUR neto. Baseline 2026-10 actualizado.
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -451,7 +451,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="51" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -613,10 +613,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>63.3</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>93.88</v>
@@ -642,7 +642,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -654,15 +654,11 @@
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -670,7 +666,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-08-02; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-08-10; sin vender → precio Ocupación</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -681,333 +677,327 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="H3" s="3" t="n">
+      <c r="F3" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>93.88</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="2" t="n">
         <v>99.5</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="2" t="n">
         <v>107.5</v>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (94€–97€)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>95.37</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>95.06999999999999</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>85.56</v>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-08-13; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>93.88</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>121.47</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>52.16</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>66.91</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (99€–102€)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>100.43</v>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (59€–63€)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n">
-        <v>100.43</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>90.39</v>
-      </c>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada alta + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-07-29; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>93.88</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>121.47</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="O4" s="3" t="n">
+        <v>61.33</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>52.16</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>75.61</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>52.16</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>66.91</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>54.47</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W4" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X4" s="2" t="n">
-        <v>75.08</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>66.44</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (57€–61€)</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>59.16</v>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>397.67</v>
-      </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="M5" s="2" t="n">
+        <v>54.01</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>54.19</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>48.77</v>
+      </c>
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr">
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W5" s="3" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="X5" s="3" t="n">
-        <v>75.08</v>
+      <c r="W5" s="2" t="n">
+        <v>46.94</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>75.61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>15.6</v>
+        <v>22.2</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>43.9</v>
+        <v>52.16</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>47.75</v>
+        <v>60.2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>50</v>
+        <v>66.91</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -1016,11 +1006,11 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (48€–49€)</t>
+          <t>P45–P60  (59€–63€)</t>
         </is>
       </c>
       <c r="M6" s="3" t="n">
-        <v>48.17</v>
+        <v>61.1</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -1028,141 +1018,239 @@
         </is>
       </c>
       <c r="O6" s="3" t="n">
-        <v>48.4</v>
+        <v>61.79</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>43.56</v>
+        <v>55.61</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>321.86</v>
+        <v>410.9</v>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+          <t>Revisar 2026-09-19; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W6" s="3" t="n">
-        <v>43.9</v>
+        <v>52.16</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>56.5</v>
+        <v>75.61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>43.56</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>321.86</v>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>2026-12-07</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C8" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Diciembre (1-19)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>131</v>
-      </c>
-      <c r="G7" s="3" t="n">
+      <c r="F8" s="3" t="n">
+        <v>119</v>
+      </c>
+      <c r="G8" s="3" t="n">
         <v>11.1</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H8" s="3" t="n">
         <v>42.03</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I8" s="3" t="n">
         <v>43.45</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>46.67</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (43€–45€)</t>
         </is>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="M8" s="3" t="n">
         <v>43.83</v>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O7" s="3" t="n">
+      <c r="O8" s="3" t="n">
         <v>44.07</v>
       </c>
-      <c r="P7" s="3" t="n">
+      <c r="P8" s="3" t="n">
         <v>39.66</v>
       </c>
-      <c r="Q7" s="3" t="n">
+      <c r="Q8" s="3" t="n">
         <v>293.07</v>
       </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="S8" s="3" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="U7" s="3" t="inlineStr">
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="V8" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W7" s="3" t="n">
+      <c r="W8" s="3" t="n">
         <v>42.03</v>
       </c>
-      <c r="X7" s="3" t="n">
+      <c r="X8" s="3" t="n">
         <v>52.74</v>
       </c>
     </row>
@@ -1590,25 +1678,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>52.08</v>
+        <v>52.16</v>
       </c>
       <c r="C11" t="n">
-        <v>55.75</v>
+        <v>55.85</v>
       </c>
       <c r="D11" t="n">
-        <v>57</v>
+        <v>58.8</v>
       </c>
       <c r="E11" t="n">
-        <v>60.1</v>
+        <v>60.2</v>
       </c>
       <c r="F11" t="n">
-        <v>61.31</v>
+        <v>63.4</v>
       </c>
       <c r="G11" t="n">
-        <v>64.81</v>
+        <v>64.83</v>
       </c>
       <c r="H11" t="n">
-        <v>66.44</v>
+        <v>66.91</v>
       </c>
       <c r="I11" t="n">
         <v>38</v>
@@ -1617,7 +1705,7 @@
         <v>92</v>
       </c>
       <c r="K11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -1769,7 +1857,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1893,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.021 (auto — vs 1.021 auto)</t>
+          <t>1.030 (auto — vs 1.030 auto)</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1905,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.021</t>
+          <t>1.030</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2122,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-29 14:07:05</t>
+          <t>2026-08-10 15:08:44</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2054,17 +2142,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.021</t>
+          <t>1.030</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.021</t>
+          <t>1.030</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva: Jorg Meissner (HMHSPXXA3A)
Mayo 2027, 3 noches, 238.86EUR. Baseline 2027-05 actualizado (374.53->613.39 income, 5->8 noches).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="51" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>70</v>
@@ -659,14 +659,10 @@
       </c>
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
+      <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-08-10; sin vender → precio Ocupación</t>
+          <t>Hueco próximo — revisar diariamente</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -701,7 +697,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>58.9</v>
@@ -793,7 +789,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>37.8</v>
@@ -889,7 +885,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>28.9</v>
@@ -918,19 +914,19 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
-        <v>54.19</v>
+        <v>53.82</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>48.77</v>
+        <v>48.44</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -985,7 +981,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>22.2</v>
@@ -1083,7 +1079,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>15.6</v>
@@ -1181,7 +1177,7 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>11.1</v>
@@ -1857,7 +1853,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2118,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-10 15:08:44</t>
+          <t>2026-08-13 09:10:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva Katja Sterzenbach (HM3JRPK3B3) + reviews Tiani Les y Dmitry Shpak
Reserva 20-24 oct 2026 (4n, 306.14EUR nrf) cubre hueco de octubre.
2 reviews 5 estrellas anadidas (369 reviews totales).
Baseline audit actualizado para 2026-10 tras el nuevo ingreso.
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -46,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE9D9"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FDE9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="43" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -591,192 +591,208 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>70</v>
+        <v>42.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>93.88</v>
+        <v>52.25</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>99.5</v>
+        <v>60.27</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>107.5</v>
+        <v>67.25</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación</t>
+          <t>Equilibrio</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>P25–P40  (94€–97€)</t>
+          <t>P45–P60  (60€–65€)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>95.37</v>
+        <v>62.42</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>95.06999999999999</v>
+        <v>62.66</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>85.56</v>
+        <v>56.39</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%) + ocupación futura alta (↑10%).</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
+          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Hueco próximo — revisar diariamente</t>
+          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>84.48999999999999</v>
+        <v>52.25</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>121.47</v>
+        <v>75.98999999999999</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>58.9</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>93.88</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>107.5</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>52.25</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>60.27</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>67.25</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>P25–P40  (94€–97€)</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>95.37</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>95.06999999999999</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>85.56</v>
-      </c>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-08-13; sin vender → bajar 5–10%</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="n">
-        <v>93.88</v>
-      </c>
-      <c r="X3" s="2" t="n">
-        <v>121.47</v>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–56€)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>54.28</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>48.85</v>
+      </c>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>47.02</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>75.98999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -789,464 +805,366 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>37.8</v>
+        <v>26.7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>52.16</v>
+        <v>52.25</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>60.2</v>
+        <v>60.27</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>66.91</v>
+        <v>67.25</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio</t>
+          <t>Ocupación</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>P45–P60  (59€–63€)</t>
+          <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>61.1</v>
+        <v>54.1</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>61.33</v>
+        <v>53.91</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>55.2</v>
+        <v>48.52</v>
       </c>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+          <t>Revisar 2026-09-19; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>52.16</v>
+        <v>47.02</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>75.61</v>
+        <v>75.98999999999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>52.16</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>60.2</v>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>66.91</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>52.25</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>60.27</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>67.25</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>P25–P40  (52€–56€)</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
-        <v>54.01</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="M5" s="3" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>48.44</v>
-      </c>
-      <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="O5" s="3" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>48.52</v>
+      </c>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W5" s="2" t="n">
-        <v>46.94</v>
-      </c>
-      <c r="X5" s="2" t="n">
-        <v>75.61</v>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-09-24; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>52.25</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>75.98999999999999</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>52.16</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>60.2</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>66.91</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (59€–63€)</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>P45–P60  (48€–49€)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O6" s="3" t="n">
-        <v>61.79</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>55.61</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>410.9</v>
-      </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="U6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-19; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="3" t="n">
-        <v>52.16</v>
-      </c>
-      <c r="X6" s="3" t="n">
-        <v>75.61</v>
+      <c r="O6" s="2" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>43.56</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>321.86</v>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>56.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-03</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-23</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre (1-19)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>42.03</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (48€–49€)</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>P45–P60  (43€–45€)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>43.83</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O7" s="3" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>43.56</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>321.86</v>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="O7" s="2" t="n">
+        <v>44.07</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>39.66</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>293.07</v>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>56.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Diciembre (1-19)</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>baja</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>116</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H8" s="3" t="n">
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n">
         <v>42.03</v>
       </c>
-      <c r="I8" s="3" t="n">
-        <v>43.45</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>46.67</v>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (43€–45€)</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>43.83</v>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>44.07</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>39.66</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>293.07</v>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S8" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="T8" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-22</t>
-        </is>
-      </c>
-      <c r="U8" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="V8" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W8" s="3" t="n">
-        <v>42.03</v>
-      </c>
-      <c r="X8" s="3" t="n">
+      <c r="X7" s="2" t="n">
         <v>52.74</v>
       </c>
     </row>
@@ -1674,25 +1592,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>52.16</v>
+        <v>52.25</v>
       </c>
       <c r="C11" t="n">
-        <v>55.85</v>
+        <v>55.95</v>
       </c>
       <c r="D11" t="n">
-        <v>58.8</v>
+        <v>60.03</v>
       </c>
       <c r="E11" t="n">
-        <v>60.2</v>
+        <v>60.27</v>
       </c>
       <c r="F11" t="n">
-        <v>63.4</v>
+        <v>64.81</v>
       </c>
       <c r="G11" t="n">
-        <v>64.83</v>
+        <v>65.08</v>
       </c>
       <c r="H11" t="n">
-        <v>66.91</v>
+        <v>67.25</v>
       </c>
       <c r="I11" t="n">
         <v>38</v>
@@ -1701,7 +1619,7 @@
         <v>92</v>
       </c>
       <c r="K11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -1853,7 +1771,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1807,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.030 (auto — vs 1.030 auto)</t>
+          <t>1.044 (auto — vs 1.044 auto)</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1819,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.030</t>
+          <t>1.044</t>
         </is>
       </c>
     </row>
@@ -2118,12 +2036,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-13 09:10:10</t>
+          <t>2026-08-31 12:48:53</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2138,17 +2056,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.030</t>
+          <t>1.044</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.030</t>
+          <t>1.044</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>